<commit_message>
Data feed from ODK setup
</commit_message>
<xml_diff>
--- a/EVD DASHBOARD/PoE_screening_data.xlsx
+++ b/EVD DASHBOARD/PoE_screening_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\genatha\Documents\Ebola SSD\Epi_Surveillance\Deliverables\PoE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="428" documentId="8_{DDDF8032-4B17-4ADF-9545-3D1D08CAE793}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E316F1E-C016-4EA3-A2D4-16EF26415137}"/>
+  <xr:revisionPtr revIDLastSave="480" documentId="8_{DDDF8032-4B17-4ADF-9545-3D1D08CAE793}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFFCF8F1-E57E-4CEE-B806-523915068E51}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Daily entry" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="209">
   <si>
     <t>Date</t>
   </si>
@@ -675,7 +675,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -732,6 +732,13 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -825,7 +832,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -852,6 +859,7 @@
     <xf numFmtId="164" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1913,91 +1921,191 @@
       <c r="I29" s="3"/>
     </row>
     <row r="30" spans="1:9">
-      <c r="A30" s="15"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
+      <c r="A30" s="15">
+        <v>46302</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" s="18">
+        <v>11378</v>
+      </c>
+      <c r="D30" s="3">
+        <v>7670</v>
+      </c>
       <c r="E30" s="13"/>
-      <c r="F30" s="3"/>
-      <c r="G30" s="3"/>
-      <c r="H30" s="3"/>
+      <c r="F30" s="3">
+        <v>0</v>
+      </c>
+      <c r="G30" s="3">
+        <v>0</v>
+      </c>
+      <c r="H30" s="3">
+        <v>0</v>
+      </c>
       <c r="I30" s="3"/>
     </row>
     <row r="31" spans="1:9">
-      <c r="A31" s="15"/>
-      <c r="B31" s="3"/>
+      <c r="A31" s="15">
+        <v>46302</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="3"/>
-      <c r="G31" s="3"/>
-      <c r="H31" s="3"/>
+      <c r="E31" s="13">
+        <v>2830</v>
+      </c>
+      <c r="F31" s="3">
+        <v>0</v>
+      </c>
+      <c r="G31" s="3">
+        <v>0</v>
+      </c>
+      <c r="H31" s="3">
+        <v>0</v>
+      </c>
       <c r="I31" s="3"/>
     </row>
     <row r="32" spans="1:9">
-      <c r="A32" s="15"/>
-      <c r="B32" s="3"/>
+      <c r="A32" s="15">
+        <v>46302</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>13</v>
+      </c>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
+      <c r="E32" s="13">
+        <v>1185</v>
+      </c>
+      <c r="F32" s="3">
+        <v>0</v>
+      </c>
+      <c r="G32" s="3">
+        <v>0</v>
+      </c>
+      <c r="H32" s="3">
+        <v>0</v>
+      </c>
       <c r="I32" s="3"/>
     </row>
     <row r="33" spans="1:9">
-      <c r="A33" s="15"/>
-      <c r="B33" s="3"/>
+      <c r="A33" s="15">
+        <v>46302</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>12</v>
+      </c>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
-      <c r="E33" s="13"/>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
+      <c r="E33" s="13">
+        <v>569</v>
+      </c>
+      <c r="F33" s="3">
+        <v>0</v>
+      </c>
+      <c r="G33" s="3">
+        <v>0</v>
+      </c>
+      <c r="H33" s="3">
+        <v>0</v>
+      </c>
       <c r="I33" s="3"/>
     </row>
     <row r="34" spans="1:9">
-      <c r="A34" s="15"/>
-      <c r="B34" s="3"/>
+      <c r="A34" s="15">
+        <v>46303</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>11</v>
+      </c>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
-      <c r="E34" s="13"/>
-      <c r="F34" s="3"/>
-      <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
+      <c r="E34" s="13">
+        <v>2540</v>
+      </c>
+      <c r="F34" s="3">
+        <v>0</v>
+      </c>
+      <c r="G34" s="3">
+        <v>0</v>
+      </c>
+      <c r="H34" s="3">
+        <v>0</v>
+      </c>
       <c r="I34" s="3"/>
     </row>
     <row r="35" spans="1:9">
-      <c r="A35" s="15"/>
-      <c r="B35" s="3"/>
+      <c r="A35" s="15">
+        <v>46303</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>12</v>
+      </c>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
-      <c r="E35" s="13"/>
-      <c r="F35" s="3"/>
-      <c r="G35" s="3"/>
-      <c r="H35" s="3"/>
+      <c r="E35" s="13">
+        <v>588</v>
+      </c>
+      <c r="F35" s="3">
+        <v>0</v>
+      </c>
+      <c r="G35" s="3">
+        <v>0</v>
+      </c>
+      <c r="H35" s="3">
+        <v>0</v>
+      </c>
       <c r="I35" s="3"/>
     </row>
     <row r="36" spans="1:9">
-      <c r="A36" s="15"/>
-      <c r="B36" s="3"/>
+      <c r="A36" s="15">
+        <v>46303</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>13</v>
+      </c>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
-      <c r="E36" s="13"/>
-      <c r="F36" s="3"/>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
+      <c r="E36" s="13">
+        <v>1305</v>
+      </c>
+      <c r="F36" s="3">
+        <v>0</v>
+      </c>
+      <c r="G36" s="3">
+        <v>0</v>
+      </c>
+      <c r="H36" s="3">
+        <v>0</v>
+      </c>
       <c r="I36" s="3"/>
     </row>
     <row r="37" spans="1:9">
-      <c r="A37" s="15"/>
-      <c r="B37" s="3"/>
-      <c r="C37" s="3"/>
-      <c r="D37" s="3"/>
+      <c r="A37" s="15">
+        <v>46303</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37" s="3">
+        <v>11792</v>
+      </c>
+      <c r="D37" s="3">
+        <v>8178</v>
+      </c>
       <c r="E37" s="13"/>
-      <c r="F37" s="3"/>
-      <c r="G37" s="3"/>
-      <c r="H37" s="3"/>
+      <c r="F37" s="3">
+        <v>0</v>
+      </c>
+      <c r="G37" s="3">
+        <v>0</v>
+      </c>
+      <c r="H37" s="3">
+        <v>0</v>
+      </c>
       <c r="I37" s="3"/>
     </row>
     <row r="38" spans="1:9">
@@ -4547,11 +4655,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="18">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
     </row>
     <row r="2" spans="1:17">
       <c r="A2" s="6" t="s">
@@ -4559,7 +4667,7 @@
       </c>
       <c r="B2" s="10">
         <f ca="1">TODAY()-14</f>
-        <v>46289</v>
+        <v>46291</v>
       </c>
       <c r="C2" s="9" t="s">
         <v>88</v>
@@ -4577,59 +4685,59 @@
       </c>
       <c r="D4" s="11">
         <f ca="1">$B$2+0</f>
-        <v>46289</v>
+        <v>46291</v>
       </c>
       <c r="E4" s="11">
         <f ca="1">$B$2+1</f>
-        <v>46290</v>
+        <v>46292</v>
       </c>
       <c r="F4" s="11">
         <f ca="1">$B$2+2</f>
-        <v>46291</v>
+        <v>46293</v>
       </c>
       <c r="G4" s="11">
         <f ca="1">$B$2+4</f>
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="H4" s="11">
         <f ca="1">$B$2+5</f>
-        <v>46294</v>
+        <v>46296</v>
       </c>
       <c r="I4" s="11">
         <f ca="1">$B$2+6</f>
-        <v>46295</v>
+        <v>46297</v>
       </c>
       <c r="J4" s="11">
         <f ca="1">$B$2+7</f>
-        <v>46296</v>
+        <v>46298</v>
       </c>
       <c r="K4" s="11">
         <f ca="1">$B$2+8</f>
-        <v>46297</v>
+        <v>46299</v>
       </c>
       <c r="L4" s="11">
         <f ca="1">$B$2+9</f>
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="M4" s="11">
         <f ca="1">$B$2+10</f>
-        <v>46299</v>
+        <v>46301</v>
       </c>
       <c r="N4" s="11">
         <f ca="1">$B$2+11</f>
-        <v>46300</v>
+        <v>46302</v>
       </c>
       <c r="O4" s="11">
         <f ca="1">$B$2+12</f>
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="P4" s="11">
         <f ca="1">$B$2+13</f>
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="Q4" s="11">
         <f ca="1">$B$2+14</f>
-        <v>46303</v>
+        <v>46305</v>
       </c>
     </row>
     <row r="5" spans="1:17" ht="15.75">
@@ -4707,11 +4815,11 @@
       </c>
       <c r="B6" s="4">
         <f t="shared" ref="B6:B43" ca="1" si="0">COUNTIF(D11:Q11,"✓")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C6" s="4">
         <f>IF(COUNTIF('Daily entry'!$B$2:$B$3001,$A11)=0,"Never",_xlfn.MAXIFS('Daily entry'!$A$2:$A$3001,'Daily entry'!$B$2:$B$3001,$A11))</f>
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="D6" s="5" t="str">
         <f ca="1">IF(COUNTIFS('Daily entry'!$A$2:$A$3001,D$4,'Daily entry'!$B$2:$B$3001,$A6)&gt;0,"✓","✗")</f>
@@ -4776,11 +4884,11 @@
       </c>
       <c r="B7" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C7" s="4">
         <f>IF(COUNTIF('Daily entry'!$B$2:$B$3001,$A12)=0,"Never",_xlfn.MAXIFS('Daily entry'!$A$2:$A$3001,'Daily entry'!$B$2:$B$3001,$A12))</f>
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="D7" s="5" t="str">
         <f ca="1">IF(COUNTIFS('Daily entry'!$A$2:$A$3001,D$4,'Daily entry'!$B$2:$B$3001,$A7)&gt;0,"✓","✗")</f>
@@ -4845,11 +4953,11 @@
       </c>
       <c r="B8" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C8" s="4">
         <f>IF(COUNTIF('Daily entry'!$B$2:$B$3001,$A13)=0,"Never",_xlfn.MAXIFS('Daily entry'!$A$2:$A$3001,'Daily entry'!$B$2:$B$3001,$A13))</f>
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="D8" s="5" t="str">
         <f ca="1">IF(COUNTIFS('Daily entry'!$A$2:$A$3001,D$4,'Daily entry'!$B$2:$B$3001,$A8)&gt;0,"✓","✗")</f>
@@ -5072,11 +5180,11 @@
       </c>
       <c r="G11" s="5" t="str">
         <f ca="1">IF(COUNTIFS('Daily entry'!$A$2:$A$3001,G$4,'Daily entry'!$B$2:$B$3001,$A11)&gt;0,"✓","✗")</f>
-        <v>✗</v>
+        <v>✓</v>
       </c>
       <c r="H11" s="5" t="str">
         <f ca="1">IF(COUNTIFS('Daily entry'!$A$2:$A$3001,H$4,'Daily entry'!$B$2:$B$3001,$A11)&gt;0,"✓","✗")</f>
-        <v>✗</v>
+        <v>✓</v>
       </c>
       <c r="I11" s="5" t="str">
         <f ca="1">IF(COUNTIFS('Daily entry'!$A$2:$A$3001,I$4,'Daily entry'!$B$2:$B$3001,$A11)&gt;0,"✓","✗")</f>
@@ -5121,11 +5229,11 @@
       </c>
       <c r="B12" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C12" s="4">
         <f>IF(COUNTIF('Daily entry'!$B$2:$B$3001,$A17)=0,"Never",_xlfn.MAXIFS('Daily entry'!$A$2:$A$3001,'Daily entry'!$B$2:$B$3001,$A17))</f>
-        <v>46301</v>
+        <v>46303</v>
       </c>
       <c r="D12" s="5" t="str">
         <f ca="1">IF(COUNTIFS('Daily entry'!$A$2:$A$3001,D$4,'Daily entry'!$B$2:$B$3001,$A12)&gt;0,"✓","✗")</f>
@@ -5141,11 +5249,11 @@
       </c>
       <c r="G12" s="5" t="str">
         <f ca="1">IF(COUNTIFS('Daily entry'!$A$2:$A$3001,G$4,'Daily entry'!$B$2:$B$3001,$A12)&gt;0,"✓","✗")</f>
-        <v>✗</v>
+        <v>✓</v>
       </c>
       <c r="H12" s="5" t="str">
         <f ca="1">IF(COUNTIFS('Daily entry'!$A$2:$A$3001,H$4,'Daily entry'!$B$2:$B$3001,$A12)&gt;0,"✓","✗")</f>
-        <v>✗</v>
+        <v>✓</v>
       </c>
       <c r="I12" s="5" t="str">
         <f ca="1">IF(COUNTIFS('Daily entry'!$A$2:$A$3001,I$4,'Daily entry'!$B$2:$B$3001,$A12)&gt;0,"✓","✗")</f>
@@ -5210,11 +5318,11 @@
       </c>
       <c r="G13" s="5" t="str">
         <f ca="1">IF(COUNTIFS('Daily entry'!$A$2:$A$3001,G$4,'Daily entry'!$B$2:$B$3001,$A13)&gt;0,"✓","✗")</f>
-        <v>✗</v>
+        <v>✓</v>
       </c>
       <c r="H13" s="5" t="str">
         <f ca="1">IF(COUNTIFS('Daily entry'!$A$2:$A$3001,H$4,'Daily entry'!$B$2:$B$3001,$A13)&gt;0,"✓","✗")</f>
-        <v>✗</v>
+        <v>✓</v>
       </c>
       <c r="I13" s="5" t="str">
         <f ca="1">IF(COUNTIFS('Daily entry'!$A$2:$A$3001,I$4,'Daily entry'!$B$2:$B$3001,$A13)&gt;0,"✓","✗")</f>
@@ -5486,11 +5594,11 @@
       </c>
       <c r="G17" s="5" t="str">
         <f ca="1">IF(COUNTIFS('Daily entry'!$A$2:$A$3001,G$4,'Daily entry'!$B$2:$B$3001,$A17)&gt;0,"✓","✗")</f>
-        <v>✗</v>
+        <v>✓</v>
       </c>
       <c r="H17" s="5" t="str">
         <f ca="1">IF(COUNTIFS('Daily entry'!$A$2:$A$3001,H$4,'Daily entry'!$B$2:$B$3001,$A17)&gt;0,"✓","✗")</f>
-        <v>✗</v>
+        <v>✓</v>
       </c>
       <c r="I17" s="5" t="str">
         <f ca="1">IF(COUNTIFS('Daily entry'!$A$2:$A$3001,I$4,'Daily entry'!$B$2:$B$3001,$A17)&gt;0,"✓","✗")</f>
@@ -12139,15 +12247,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000D45862254BD58479CB6D95C1D4AAE6A" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="dc7916497a1fd6819727e31f7bf64d18">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="761af89e-1749-4001-a5ec-3f4afda2eb63" xmlns:ns3="de11a23f-3553-4745-b513-83632ef1acf3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fdb4f5cd6010e2afd34077ea8abb84d1" ns2:_="" ns3:_="">
     <xsd:import namespace="761af89e-1749-4001-a5ec-3f4afda2eb63"/>
@@ -12402,14 +12501,23 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8807BD22-57E1-4C10-A3B5-4820048C45D4}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06A5175C-0130-4752-B62F-1E389FE5048F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFF9C6AB-A604-4632-B100-1FAF3710D944}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFF9C6AB-A604-4632-B100-1FAF3710D944}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06A5175C-0130-4752-B62F-1E389FE5048F}"/>
 </file>
</xml_diff>